<commit_message>
Add interest-only period to UW model debt
- New "Interest-Only Period (years)" assumption. Debt tab now shows interest-only
  vs. amortizing annual debt service, the actual Year-1 DSCR and the amortizing
  (stress) DSCR, and an exit balance that stays at the full loan through IO then
  amortizes.
- Returns applies per-year debt service (interest-only for years 1..IO, amortizing
  after) and the Sensitivity backing calcs do the same, so every IRR reflects the
  IO structure.

Illustrative deal (2-yr IO): DSCR 1.64x actual / 1.41x amortizing; levered IRR
15.5%, cash-on-cash 7.6% (front-loaded by the IO period).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Agyvs8LTH6G2FjDZg6YMxz
</commit_message>
<xml_diff>
--- a/templates/UW_Model_Template.xlsx
+++ b/templates/UW_Model_Template.xlsx
@@ -754,7 +754,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="25" customHeight="1">
+    <row r="14" ht="37.5" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>Debt</t>
@@ -762,7 +762,7 @@
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Sizes &amp; amortizes the loan: annual debt service, DSCR, debt yield, and the loan payoff balance in the hold year.</t>
+          <t>Sizes the loan and supports an INTEREST-ONLY period: interest-only debt service for the first N years, then the amortizing payment. Shows both the actual Year-1 DSCR and the amortizing (stress) DSCR, debt yield, and the exit payoff balance (full loan through IO, amortizing after).</t>
         </is>
       </c>
     </row>
@@ -1381,103 +1381,103 @@
         </is>
       </c>
       <c r="B23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="C23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="M23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="N23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="O23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="P23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Q23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="R23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="S23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="T23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="U23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="V23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="W23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="X23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Y23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Z23" s="12">
-        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-'Debt'!$B$9,0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(1&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)-IF(1&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(1='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^0+'Renovation'!B$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^0)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>
@@ -1488,103 +1488,103 @@
         </is>
       </c>
       <c r="B24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="C24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="M24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="N24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="O24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="P24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Q24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="R24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="S24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="T24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="U24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="V24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="W24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="X24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Y24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Z24" s="12">
-        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-'Debt'!$B$9,0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(2&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)-IF(2&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(2='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^1+'Renovation'!C$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^1)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>
@@ -1595,103 +1595,103 @@
         </is>
       </c>
       <c r="B25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="C25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="M25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="N25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="O25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="P25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Q25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="R25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="S25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="T25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="U25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="V25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="W25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="X25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Y25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Z25" s="12">
-        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-'Debt'!$B$9,0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(3&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)-IF(3&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(3='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^2+'Renovation'!D$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^2)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>
@@ -1702,103 +1702,103 @@
         </is>
       </c>
       <c r="B26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="C26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="M26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="N26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="O26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="P26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Q26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="R26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="S26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="T26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="U26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="V26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="W26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="X26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Y26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Z26" s="12">
-        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-'Debt'!$B$9,0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(4&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)-IF(4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(4='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^3+'Renovation'!E$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^3)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>
@@ -1809,103 +1809,103 @@
         </is>
       </c>
       <c r="B27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="C27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="M27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="N27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="O27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="P27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Q27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="R27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="S27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="T27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="U27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="V27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="W27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="X27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Y27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Z27" s="12">
-        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-'Debt'!$B$9,0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(5&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)-IF(5&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(5='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^4+'Renovation'!F$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^4)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>
@@ -1916,103 +1916,103 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="M28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="N28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="O28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="P28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Q28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="R28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="S28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="T28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="U28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="V28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="W28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="X28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Y28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Z28" s="12">
-        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-'Debt'!$B$9,0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(6&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)-IF(6&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(6='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^5+'Renovation'!G$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^5)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>
@@ -2023,103 +2023,103 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="M29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="N29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="O29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="P29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Q29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="R29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="S29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="T29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="U29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="V29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="W29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="X29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Y29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Z29" s="12">
-        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-'Debt'!$B$9,0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(7&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)-IF(7&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(7='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^6+'Renovation'!H$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^6)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>
@@ -2130,103 +2130,103 @@
         </is>
       </c>
       <c r="B30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="M30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="N30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="O30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="P30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Q30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="R30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="S30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="T30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="U30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="V30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="W30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="X30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Y30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Z30" s="12">
-        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-'Debt'!$B$9,0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(8&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)-IF(8&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(8='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^7+'Renovation'!I$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^7)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>
@@ -2237,103 +2237,103 @@
         </is>
       </c>
       <c r="B31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="C31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="M31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="N31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="O31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="P31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Q31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="R31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="S31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="T31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="U31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="V31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="W31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="X31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Y31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Z31" s="12">
-        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-'Debt'!$B$9,0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(9&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)-IF(9&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(9='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^8+'Renovation'!J$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^8)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>
@@ -2344,103 +2344,103 @@
         </is>
       </c>
       <c r="B32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+B$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/B$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="C32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+C$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/C$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+D$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/D$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+E$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/E$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+F$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/F$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+G$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/G$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+H$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/H$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+I$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/I$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+J$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/J$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+K$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/K$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+L$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/L$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="M32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+M$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/M$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="N32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+N$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/N$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="O32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+O$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/O$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="P32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+P$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/P$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Q32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Q$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/Q$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="R32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+R$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/R$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="S32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+S$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/S$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="T32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+T$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/T$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="U32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+U$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/U$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="V32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+V$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/V$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="W32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+W$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/W$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="X32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+X$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/X$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Y32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Y$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/Y$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="Z32" s="12">
-        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-'Debt'!$B$9,0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$12,0)</f>
+        <f>IF(10&lt;='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)-IF(10&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)+IF(10='Assumptions'!$B$8,('P&amp;L'!$C$10*(1+Z$20)^9+'Renovation'!K$18-'P&amp;L'!$C$23*(1+'Assumptions'!$B$15)^9)/Z$21*(1-'Assumptions'!$B$10)-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>
@@ -2565,7 +2565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2808,14 +2808,29 @@
     <row r="25">
       <c r="A25" s="8" t="inlineStr">
         <is>
+          <t>Interest-Only Period (years)</t>
+        </is>
+      </c>
+      <c r="B25" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="C25" s="10" t="inlineStr">
+        <is>
+          <t>Interest-only years before amortization begins (0 = fully amortizing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
           <t>Renovation Budget (auto)</t>
         </is>
       </c>
-      <c r="B25" s="19">
+      <c r="B26" s="19">
         <f>'Renovation'!$E$9</f>
         <v/>
       </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>Totals up from the Renovation tab scope.</t>
         </is>
@@ -4623,7 +4638,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C12"/>
+  <dimension ref="A1:C15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4679,86 +4694,139 @@
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Hold Period (years)</t>
+          <t>Interest-Only Period (years)</t>
         </is>
       </c>
       <c r="B7" s="11">
-        <f>'Assumptions'!$B$8</f>
-        <v/>
+        <f>'Assumptions'!$B$25</f>
+        <v/>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>Interest-only years before amortization.</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Monthly Payment</t>
-        </is>
-      </c>
-      <c r="B8" s="35">
+          <t>Hold Period (years)</t>
+        </is>
+      </c>
+      <c r="B8" s="11">
+        <f>'Assumptions'!$B$8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Monthly Amortizing Payment</t>
+        </is>
+      </c>
+      <c r="B9" s="35">
         <f>PMT(B5/12,B6*12,-B4)</f>
         <v/>
       </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>Standard amortizing payment.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="21" t="inlineStr">
-        <is>
-          <t>Annual Debt Service</t>
-        </is>
-      </c>
-      <c r="B9" s="36">
-        <f>B8*12</f>
-        <v/>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>Payment once amortization begins.</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>DSCR (Year-1 NOI)</t>
-        </is>
-      </c>
-      <c r="B10" s="37">
-        <f>'Pro Forma'!$B$8/B9</f>
+          <t>Annual Debt Service — Interest-Only</t>
+        </is>
+      </c>
+      <c r="B10" s="12">
+        <f>B4*B5</f>
         <v/>
       </c>
       <c r="C10" s="10" t="inlineStr">
         <is>
-          <t>NOI / debt service. Lenders want &gt;= ~1.25x.</t>
+          <t>Years 1..IO: interest only.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Debt Yield (Year-1 NOI)</t>
-        </is>
-      </c>
-      <c r="B11" s="32">
-        <f>'Pro Forma'!$B$8/B4</f>
+      <c r="A11" s="21" t="inlineStr">
+        <is>
+          <t>Annual Debt Service — Amortizing</t>
+        </is>
+      </c>
+      <c r="B11" s="36">
+        <f>B9*12</f>
         <v/>
       </c>
       <c r="C11" s="10" t="inlineStr">
         <is>
-          <t>NOI / loan.</t>
+          <t>After the IO period.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="inlineStr">
         <is>
+          <t>DSCR — Year 1 (actual)</t>
+        </is>
+      </c>
+      <c r="B12" s="37">
+        <f>'Pro Forma'!$B$8/IF(1&lt;=B7,B10,B11)</f>
+        <v/>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>On the actual Year-1 payment (IO if applicable).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>DSCR — Amortizing (stress)</t>
+        </is>
+      </c>
+      <c r="B13" s="37">
+        <f>'Pro Forma'!$B$8/B11</f>
+        <v/>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>Lender stress at the amortizing payment. Want &gt;= ~1.25x.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Debt Yield (Year-1 NOI)</t>
+        </is>
+      </c>
+      <c r="B14" s="32">
+        <f>'Pro Forma'!$B$8/B4</f>
+        <v/>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>NOI / loan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
           <t>Loan Balance at Exit</t>
         </is>
       </c>
-      <c r="B12" s="12">
-        <f>B8*(1-(1+B5/12)^-(B6*12-B7*12))/(B5/12)</f>
-        <v/>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>Remaining principal in the hold year.</t>
+      <c r="B15" s="12">
+        <f>IF(B8&lt;=B7,B4,B9*(1-(1+B5/12)^-(B6*12-(B8-B7)*12))/(B5/12))</f>
+        <v/>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Full loan through IO; amortizes after.</t>
         </is>
       </c>
     </row>
@@ -4956,43 +5024,43 @@
         </is>
       </c>
       <c r="C6" s="12">
-        <f>IF(AND(C$4&gt;=1,C$4&lt;='Assumptions'!$B$8),-'Debt'!$B$9,0)</f>
+        <f>IF(AND(C$4&gt;=1,C$4&lt;='Assumptions'!$B$8),-IF(C$4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)</f>
         <v/>
       </c>
       <c r="D6" s="12">
-        <f>IF(AND(D$4&gt;=1,D$4&lt;='Assumptions'!$B$8),-'Debt'!$B$9,0)</f>
+        <f>IF(AND(D$4&gt;=1,D$4&lt;='Assumptions'!$B$8),-IF(D$4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)</f>
         <v/>
       </c>
       <c r="E6" s="12">
-        <f>IF(AND(E$4&gt;=1,E$4&lt;='Assumptions'!$B$8),-'Debt'!$B$9,0)</f>
+        <f>IF(AND(E$4&gt;=1,E$4&lt;='Assumptions'!$B$8),-IF(E$4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)</f>
         <v/>
       </c>
       <c r="F6" s="12">
-        <f>IF(AND(F$4&gt;=1,F$4&lt;='Assumptions'!$B$8),-'Debt'!$B$9,0)</f>
+        <f>IF(AND(F$4&gt;=1,F$4&lt;='Assumptions'!$B$8),-IF(F$4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)</f>
         <v/>
       </c>
       <c r="G6" s="12">
-        <f>IF(AND(G$4&gt;=1,G$4&lt;='Assumptions'!$B$8),-'Debt'!$B$9,0)</f>
+        <f>IF(AND(G$4&gt;=1,G$4&lt;='Assumptions'!$B$8),-IF(G$4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)</f>
         <v/>
       </c>
       <c r="H6" s="12">
-        <f>IF(AND(H$4&gt;=1,H$4&lt;='Assumptions'!$B$8),-'Debt'!$B$9,0)</f>
+        <f>IF(AND(H$4&gt;=1,H$4&lt;='Assumptions'!$B$8),-IF(H$4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)</f>
         <v/>
       </c>
       <c r="I6" s="12">
-        <f>IF(AND(I$4&gt;=1,I$4&lt;='Assumptions'!$B$8),-'Debt'!$B$9,0)</f>
+        <f>IF(AND(I$4&gt;=1,I$4&lt;='Assumptions'!$B$8),-IF(I$4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)</f>
         <v/>
       </c>
       <c r="J6" s="12">
-        <f>IF(AND(J$4&gt;=1,J$4&lt;='Assumptions'!$B$8),-'Debt'!$B$9,0)</f>
+        <f>IF(AND(J$4&gt;=1,J$4&lt;='Assumptions'!$B$8),-IF(J$4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)</f>
         <v/>
       </c>
       <c r="K6" s="12">
-        <f>IF(AND(K$4&gt;=1,K$4&lt;='Assumptions'!$B$8),-'Debt'!$B$9,0)</f>
+        <f>IF(AND(K$4&gt;=1,K$4&lt;='Assumptions'!$B$8),-IF(K$4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)</f>
         <v/>
       </c>
       <c r="L6" s="12">
-        <f>IF(AND(L$4&gt;=1,L$4&lt;='Assumptions'!$B$8),-'Debt'!$B$9,0)</f>
+        <f>IF(AND(L$4&gt;=1,L$4&lt;='Assumptions'!$B$8),-IF(L$4&lt;='Assumptions'!$B$25,'Debt'!$B$10,'Debt'!$B$11),0)</f>
         <v/>
       </c>
     </row>
@@ -5144,43 +5212,43 @@
         </is>
       </c>
       <c r="C10" s="12">
-        <f>IF(C$4='Assumptions'!$B$8,-'Debt'!$B$12,0)</f>
+        <f>IF(C$4='Assumptions'!$B$8,-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="D10" s="12">
-        <f>IF(D$4='Assumptions'!$B$8,-'Debt'!$B$12,0)</f>
+        <f>IF(D$4='Assumptions'!$B$8,-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="E10" s="12">
-        <f>IF(E$4='Assumptions'!$B$8,-'Debt'!$B$12,0)</f>
+        <f>IF(E$4='Assumptions'!$B$8,-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="F10" s="12">
-        <f>IF(F$4='Assumptions'!$B$8,-'Debt'!$B$12,0)</f>
+        <f>IF(F$4='Assumptions'!$B$8,-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="G10" s="12">
-        <f>IF(G$4='Assumptions'!$B$8,-'Debt'!$B$12,0)</f>
+        <f>IF(G$4='Assumptions'!$B$8,-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="H10" s="12">
-        <f>IF(H$4='Assumptions'!$B$8,-'Debt'!$B$12,0)</f>
+        <f>IF(H$4='Assumptions'!$B$8,-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="I10" s="12">
-        <f>IF(I$4='Assumptions'!$B$8,-'Debt'!$B$12,0)</f>
+        <f>IF(I$4='Assumptions'!$B$8,-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="J10" s="12">
-        <f>IF(J$4='Assumptions'!$B$8,-'Debt'!$B$12,0)</f>
+        <f>IF(J$4='Assumptions'!$B$8,-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="K10" s="12">
-        <f>IF(K$4='Assumptions'!$B$8,-'Debt'!$B$12,0)</f>
+        <f>IF(K$4='Assumptions'!$B$8,-'Debt'!$B$15,0)</f>
         <v/>
       </c>
       <c r="L10" s="12">
-        <f>IF(L$4='Assumptions'!$B$8,-'Debt'!$B$12,0)</f>
+        <f>IF(L$4='Assumptions'!$B$8,-'Debt'!$B$15,0)</f>
         <v/>
       </c>
     </row>

</xml_diff>